<commit_message>
Section 27: OKCR pull pipeline + status update (egress blocked)
API key + APPROVE_OKCR_DOWNLOADS=true received, but okcountyrecords.com is
blocked by the environment egress allowlist (HTTP 403; pypi/github reachable).
No records downloadable here.

- Added scripts/okcr_pull.py: idempotent dry-run cost estimate + Priority-1
  image pulls, reads key from env only, never logs/commits secrets.
- Added .env.example (placeholders only).
- Updated API/OCR log, approval manifest, QA row, and workbook Change Log to
  document the attempt. No key/secret written to any output (verified).
</commit_message>
<xml_diff>
--- a/title_research/Section27_11N_25W/deliverables/11N_25W_27_Beckham_Co_Diversified_Cursory_Report_FULLY_UPDATED.xlsx
+++ b/title_research/Section27_11N_25W/deliverables/11N_25W_27_Beckham_Co_Diversified_Cursory_Report_FULLY_UPDATED.xlsx
@@ -10223,7 +10223,7 @@
       </c>
       <c r="C10" s="141" t="inlineStr">
         <is>
-          <t>Not present in provided index and no OKCR API access; carried as cited and flagged in Gap List #2.</t>
+          <t>Key+approval supplied but okcountyrecords.com is blocked by the environment egress allowlist (HTTP 403); not downloadable here. Carried as cited; run scripts/okcr_pull.py where the host is reachable. Flagged Gap #2.</t>
         </is>
       </c>
     </row>
@@ -10341,7 +10341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="120" customWidth="1" style="41" min="1" max="1"/>
@@ -10463,6 +10463,34 @@
       <c r="A19" s="143" t="inlineStr">
         <is>
           <t>- Diversified apparent WI unchanged at 0.700520833 (448.333333/640); residual 0.299479167 (191.666667/640); section ties to 640 ac / 1.000000 WI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="143" t="inlineStr">
+        <is>
+          <t>--- 2026-06-08 OKCR download attempt ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="143" t="inlineStr">
+        <is>
+          <t>- API key supplied and APPROVE_OKCR_DOWNLOADS=true set. Egress test: okcountyrecords.com returns HTTP 403 from the environment proxy (host not on the sandbox allowlist; pypi/github reachable, okcountyrecords/example.com blocked).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="143" t="inlineStr">
+        <is>
+          <t>- No records downloadable in this environment. Runnable pull pipeline scripts/okcr_pull.py delivered for execution where the host is reachable (dry-run cost estimate then idempotent Priority-1 pulls).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="143" t="inlineStr">
+        <is>
+          <t>- 2017-2026 corporate assignment chain remains carried-as-cited / unverified pending those pulls. No key/secret written to any output.</t>
         </is>
       </c>
     </row>

</xml_diff>